<commit_message>
ver problemas de male
</commit_message>
<xml_diff>
--- a/Data/Data_Raw/Country codes & metadata/metadata_new.xlsx
+++ b/Data/Data_Raw/Country codes & metadata/metadata_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/florenciaruiz/Downloads/Data-Portal-Brief-Generator/Data/Data_Raw/Country codes &amp; metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1ADB30A-BF61-964D-AAA0-A806BBD5F1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CDF620-C902-0341-A8AD-4AA376CBE2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="1520" windowWidth="23660" windowHeight="16720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="1520" windowWidth="23660" windowHeight="16720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5308,7 +5308,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:31" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A13" s="72" t="s">
         <v>150</v>
       </c>
@@ -5376,7 +5376,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="14" spans="1:31" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A14" s="72" t="s">
         <v>157</v>
       </c>
@@ -8620,7 +8620,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="55" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>449</v>
       </c>
@@ -8858,7 +8858,7 @@
       <c r="BA57"/>
       <c r="BB57"/>
     </row>
-    <row r="58" spans="1:54" s="36" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:54" s="36" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="36" t="s">
         <v>471</v>
       </c>
@@ -8965,7 +8965,7 @@
       <c r="BA58" s="5"/>
       <c r="BB58" s="5"/>
     </row>
-    <row r="59" spans="1:54" s="36" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:54" s="36" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="36" t="s">
         <v>482</v>
       </c>
@@ -9224,7 +9224,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="62" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>508</v>
       </c>
@@ -9292,7 +9292,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="63" spans="1:54" s="36" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:54" s="36" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="36" t="s">
         <v>515</v>
       </c>
@@ -9399,7 +9399,7 @@
       <c r="BA63" s="5"/>
       <c r="BB63" s="5"/>
     </row>
-    <row r="64" spans="1:54" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:54" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
         <v>527</v>
       </c>
@@ -9474,7 +9474,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="65" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>537</v>
       </c>
@@ -9551,7 +9551,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="66" spans="1:54" s="31" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:54" s="31" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="31" t="s">
         <v>545</v>
       </c>
@@ -9655,7 +9655,7 @@
       <c r="BA66"/>
       <c r="BB66"/>
     </row>
-    <row r="67" spans="1:54" s="5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:54" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
         <v>555</v>
       </c>
@@ -11440,7 +11440,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="93" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>748</v>
       </c>

</xml_diff>